<commit_message>
Update calendar: S1-12 Neo4j blog → Done
</commit_message>
<xml_diff>
--- a/Calendar/PMG_Content_Calendar_v3.xlsx
+++ b/Calendar/PMG_Content_Calendar_v3.xlsx
@@ -2359,9 +2359,9 @@
           <t>Graph-Native Supply Chain Risk — A Neo4j Perspective [Co-marketing]</t>
         </is>
       </c>
-      <c r="F30" s="60" t="inlineStr">
-        <is>
-          <t>On Hold</t>
+      <c r="F30" s="76" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G30" s="55" t="inlineStr">
@@ -4653,6 +4653,7 @@
         </is>
       </c>
     </row>
+    <row r="71"/>
     <row r="72" ht="15" customHeight="1" s="44">
       <c r="A72" s="64" t="inlineStr">
         <is>
@@ -7980,14 +7981,22 @@
           <t>Graph-Native Supply Chain Risk — A Neo4j Perspective [Co-marketing]</t>
         </is>
       </c>
-      <c r="E29" s="60" t="inlineStr">
-        <is>
-          <t>On Hold</t>
+      <c r="E29" s="76" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F29" s="55" t="n"/>
-      <c r="G29" s="55" t="n"/>
-      <c r="H29" s="55" t="n"/>
+      <c r="G29" s="55" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="H29" s="55" t="inlineStr">
+        <is>
+          <t>https://www.ecocomitychain.ai/blog/posts/graph-native-supply-chain-risk-neo4j/</t>
+        </is>
+      </c>
       <c r="I29" s="55" t="inlineStr">
         <is>
           <t>~1,000 words</t>

</xml_diff>